<commit_message>
Reverted to commit b87ce5700255f34a52eba057598b8be8b6bb0243
</commit_message>
<xml_diff>
--- a/public/ezhliha_import_template_v2.xlsx
+++ b/public/ezhliha_import_template_v2.xlsx
@@ -1841,7 +1841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -1850,7 +1850,6 @@
     <col width="35" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1884,19 +1883,11 @@
           <t>الترتيب</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>المدينة *</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="1">
     <dataValidation sqref="A2:A1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="قيمة غير صحيحة" error="اختر مزوداً من القائمة" type="list">
       <formula1>=Providers</formula1>
-    </dataValidation>
-    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"الرياض,جدة,مكة المكرمة,المدينة المنورة,الدمام,الخبر"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>